<commit_message>
Add original circuits to discovery replay workbook
</commit_message>
<xml_diff>
--- a/experiments/discovery_scalar_mma_replay_20260831/discovery_scalar_mma_replay_20260831.xlsx
+++ b/experiments/discovery_scalar_mma_replay_20260831/discovery_scalar_mma_replay_20260831.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="20">
   <si>
     <t xml:space="preserve">Benchmark</t>
   </si>
@@ -40,25 +40,46 @@
     <t xml:space="preserve">Mismatches</t>
   </si>
   <si>
+    <t xml:space="preserve">Status / note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">netcard original</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N/A - production path did not invoke deviation discovery</t>
+  </si>
+  <si>
     <t xml:space="preserve">netcard d40</t>
   </si>
   <si>
+    <t xml:space="preserve">Measured</t>
+  </si>
+  <si>
     <t xml:space="preserve">netcard d50</t>
   </si>
   <si>
+    <t xml:space="preserve">leon2 original</t>
+  </si>
+  <si>
     <t xml:space="preserve">leon2 d40</t>
   </si>
   <si>
     <t xml:space="preserve">leon2 d50</t>
   </si>
   <si>
+    <t xml:space="preserve">leon3mp original</t>
+  </si>
+  <si>
     <t xml:space="preserve">leon3mp d40</t>
   </si>
   <si>
     <t xml:space="preserve">leon3mp d50</t>
   </si>
   <si>
-    <t xml:space="preserve">Aggregate</t>
+    <t xml:space="preserve">Aggregate (measured dense cases only)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All fingerprints matched</t>
   </si>
 </sst>
 </file>
@@ -260,15 +281,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.41"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18.96"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="8.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="46.65"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -290,145 +312,211 @@
       <c r="F1" s="0" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="0" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="0" t="n">
-        <v>16.198</v>
-      </c>
-      <c r="C2" s="0" t="n">
-        <v>16.062</v>
-      </c>
-      <c r="D2" s="0" t="n">
-        <v>0.843</v>
+        <v>7</v>
       </c>
       <c r="E2" s="0" t="n">
-        <v>315</v>
+        <v>0</v>
       </c>
       <c r="F2" s="0" t="n">
         <v>0</v>
+      </c>
+      <c r="G2" s="0" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B3" s="0" t="n">
-        <v>21.829</v>
+        <v>16.198</v>
       </c>
       <c r="C3" s="0" t="n">
-        <v>21.44</v>
+        <v>16.062</v>
       </c>
       <c r="D3" s="0" t="n">
-        <v>1.815</v>
+        <v>0.843</v>
       </c>
       <c r="E3" s="0" t="n">
-        <v>404</v>
+        <v>315</v>
       </c>
       <c r="F3" s="0" t="n">
         <v>0</v>
+      </c>
+      <c r="G3" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B4" s="0" t="n">
-        <v>1.67</v>
+        <v>21.829</v>
       </c>
       <c r="C4" s="0" t="n">
-        <v>1.619</v>
+        <v>21.44</v>
       </c>
       <c r="D4" s="0" t="n">
-        <v>3.2</v>
+        <v>1.815</v>
       </c>
       <c r="E4" s="0" t="n">
-        <v>28</v>
+        <v>404</v>
       </c>
       <c r="F4" s="0" t="n">
         <v>0</v>
+      </c>
+      <c r="G4" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="0" t="n">
-        <v>18.568</v>
-      </c>
-      <c r="C5" s="0" t="n">
-        <v>18.428</v>
-      </c>
-      <c r="D5" s="0" t="n">
-        <v>0.764</v>
+        <v>12</v>
       </c>
       <c r="E5" s="0" t="n">
-        <v>356</v>
+        <v>0</v>
       </c>
       <c r="F5" s="0" t="n">
         <v>0</v>
+      </c>
+      <c r="G5" s="0" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="C6" s="0" t="n">
+        <v>1.619</v>
+      </c>
+      <c r="D6" s="0" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E6" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="F6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="0" t="s">
         <v>10</v>
-      </c>
-      <c r="B6" s="0" t="n">
-        <v>4.55</v>
-      </c>
-      <c r="C6" s="0" t="n">
-        <v>4.412</v>
-      </c>
-      <c r="D6" s="0" t="n">
-        <v>3.135</v>
-      </c>
-      <c r="E6" s="0" t="n">
-        <v>78</v>
-      </c>
-      <c r="F6" s="0" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B7" s="0" t="n">
-        <v>16.163</v>
+        <v>18.568</v>
       </c>
       <c r="C7" s="0" t="n">
-        <v>15.866</v>
+        <v>18.428</v>
       </c>
       <c r="D7" s="0" t="n">
-        <v>1.872</v>
+        <v>0.764</v>
       </c>
       <c r="E7" s="0" t="n">
-        <v>305</v>
+        <v>356</v>
       </c>
       <c r="F7" s="0" t="n">
         <v>0</v>
+      </c>
+      <c r="G7" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="E8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="0" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="C9" s="0" t="n">
+        <v>4.412</v>
+      </c>
+      <c r="D9" s="0" t="n">
+        <v>3.135</v>
+      </c>
+      <c r="E9" s="0" t="n">
+        <v>78</v>
+      </c>
+      <c r="F9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="0" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>16.163</v>
+      </c>
+      <c r="C10" s="0" t="n">
+        <v>15.866</v>
+      </c>
+      <c r="D10" s="0" t="n">
+        <v>1.872</v>
+      </c>
+      <c r="E10" s="0" t="n">
+        <v>305</v>
+      </c>
+      <c r="F10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="0" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="0" t="n">
         <v>78.979</v>
       </c>
-      <c r="C8" s="0" t="n">
+      <c r="C11" s="0" t="n">
         <v>77.826</v>
       </c>
-      <c r="D8" s="0" t="n">
+      <c r="D11" s="0" t="n">
         <v>1.48</v>
       </c>
-      <c r="E8" s="0" t="n">
+      <c r="E11" s="0" t="n">
         <v>1486</v>
       </c>
-      <c r="F8" s="0" t="n">
-        <v>0</v>
+      <c r="F11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="0" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correct discovery replay workbook with forced measurements
</commit_message>
<xml_diff>
--- a/experiments/discovery_scalar_mma_replay_20260831/discovery_scalar_mma_replay_20260831.xlsx
+++ b/experiments/discovery_scalar_mma_replay_20260831/discovery_scalar_mma_replay_20260831.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="21">
   <si>
     <t xml:space="preserve">Benchmark</t>
   </si>
@@ -40,21 +40,24 @@
     <t xml:space="preserve">Mismatches</t>
   </si>
   <si>
+    <t xml:space="preserve">Discovered pairs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maximum active paths</t>
+  </si>
+  <si>
     <t xml:space="preserve">Status / note</t>
   </si>
   <si>
     <t xml:space="preserve">netcard original</t>
   </si>
   <si>
-    <t xml:space="preserve">N/A - production path did not invoke deviation discovery</t>
+    <t xml:space="preserve">Forced identical-work discovery replay</t>
   </si>
   <si>
     <t xml:space="preserve">netcard d40</t>
   </si>
   <si>
-    <t xml:space="preserve">Measured</t>
-  </si>
-  <si>
     <t xml:space="preserve">netcard d50</t>
   </si>
   <si>
@@ -76,10 +79,10 @@
     <t xml:space="preserve">leon3mp d50</t>
   </si>
   <si>
-    <t xml:space="preserve">Aggregate (measured dense cases only)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All fingerprints matched</t>
+    <t xml:space="preserve">Aggregate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All fingerprints matched; K=100000</t>
   </si>
 </sst>
 </file>
@@ -281,16 +284,18 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.81"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.41"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18.96"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="8.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="46.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="19.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="32.45"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -315,208 +320,301 @@
       <c r="G1" s="0" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>7</v>
+        <v>9</v>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1.347</v>
+      </c>
+      <c r="C2" s="0" t="n">
+        <v>1.313</v>
+      </c>
+      <c r="D2" s="0" t="n">
+        <v>2.557</v>
       </c>
       <c r="E2" s="0" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F2" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="0" t="s">
-        <v>8</v>
+      <c r="G2" s="0" t="n">
+        <v>96220</v>
+      </c>
+      <c r="H2" s="0" t="n">
+        <v>75952</v>
+      </c>
+      <c r="I2" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B3" s="0" t="n">
-        <v>16.198</v>
+        <v>2.042</v>
       </c>
       <c r="C3" s="0" t="n">
-        <v>16.062</v>
+        <v>1.935</v>
       </c>
       <c r="D3" s="0" t="n">
-        <v>0.843</v>
+        <v>5.521</v>
       </c>
       <c r="E3" s="0" t="n">
-        <v>315</v>
+        <v>34</v>
       </c>
       <c r="F3" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="G3" s="0" t="n">
+        <v>15511</v>
+      </c>
+      <c r="H3" s="0" t="n">
+        <v>56720</v>
+      </c>
+      <c r="I3" s="0" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B4" s="0" t="n">
-        <v>21.829</v>
+        <v>2.751</v>
       </c>
       <c r="C4" s="0" t="n">
-        <v>21.44</v>
+        <v>2.598</v>
       </c>
       <c r="D4" s="0" t="n">
-        <v>1.815</v>
+        <v>5.892</v>
       </c>
       <c r="E4" s="0" t="n">
-        <v>404</v>
+        <v>38</v>
       </c>
       <c r="F4" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="G4" s="0" t="n">
+        <v>41207</v>
+      </c>
+      <c r="H4" s="0" t="n">
+        <v>176000</v>
+      </c>
+      <c r="I4" s="0" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>1.497</v>
+      </c>
+      <c r="C5" s="0" t="n">
+        <v>1.477</v>
+      </c>
+      <c r="D5" s="0" t="n">
+        <v>1.334</v>
       </c>
       <c r="E5" s="0" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="F5" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="0" t="s">
-        <v>8</v>
+      <c r="G5" s="0" t="n">
+        <v>56969</v>
+      </c>
+      <c r="H5" s="0" t="n">
+        <v>35131</v>
+      </c>
+      <c r="I5" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B6" s="0" t="n">
-        <v>1.67</v>
+        <v>2.286</v>
       </c>
       <c r="C6" s="0" t="n">
-        <v>1.619</v>
+        <v>2.194</v>
       </c>
       <c r="D6" s="0" t="n">
-        <v>3.2</v>
+        <v>4.17</v>
       </c>
       <c r="E6" s="0" t="n">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="F6" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="0" t="s">
+      <c r="G6" s="0" t="n">
+        <v>18734</v>
+      </c>
+      <c r="H6" s="0" t="n">
+        <v>102757</v>
+      </c>
+      <c r="I6" s="0" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B7" s="0" t="n">
-        <v>18.568</v>
+        <v>2.046</v>
       </c>
       <c r="C7" s="0" t="n">
-        <v>18.428</v>
+        <v>1.989</v>
       </c>
       <c r="D7" s="0" t="n">
-        <v>0.764</v>
+        <v>2.878</v>
       </c>
       <c r="E7" s="0" t="n">
-        <v>356</v>
+        <v>35</v>
       </c>
       <c r="F7" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="0" t="s">
+      <c r="G7" s="0" t="n">
+        <v>68799</v>
+      </c>
+      <c r="H7" s="0" t="n">
+        <v>61967</v>
+      </c>
+      <c r="I7" s="0" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>2.369</v>
+      </c>
+      <c r="C8" s="0" t="n">
+        <v>2.388</v>
+      </c>
+      <c r="D8" s="0" t="n">
+        <v>-0.805</v>
       </c>
       <c r="E8" s="0" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="F8" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="0" t="s">
-        <v>8</v>
+      <c r="G8" s="0" t="n">
+        <v>132875</v>
+      </c>
+      <c r="H8" s="0" t="n">
+        <v>61604</v>
+      </c>
+      <c r="I8" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B9" s="0" t="n">
-        <v>4.55</v>
+        <v>2.291</v>
       </c>
       <c r="C9" s="0" t="n">
-        <v>4.412</v>
+        <v>2.228</v>
       </c>
       <c r="D9" s="0" t="n">
-        <v>3.135</v>
+        <v>2.858</v>
       </c>
       <c r="E9" s="0" t="n">
-        <v>78</v>
+        <v>38</v>
       </c>
       <c r="F9" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="0" t="s">
+      <c r="G9" s="0" t="n">
+        <v>71117</v>
+      </c>
+      <c r="H9" s="0" t="n">
+        <v>103505</v>
+      </c>
+      <c r="I9" s="0" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B10" s="0" t="n">
-        <v>16.163</v>
+        <v>2.06</v>
       </c>
       <c r="C10" s="0" t="n">
-        <v>15.866</v>
+        <v>1.953</v>
       </c>
       <c r="D10" s="0" t="n">
-        <v>1.872</v>
+        <v>5.46</v>
       </c>
       <c r="E10" s="0" t="n">
-        <v>305</v>
+        <v>33</v>
       </c>
       <c r="F10" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="0" t="s">
+      <c r="G10" s="0" t="n">
+        <v>8721</v>
+      </c>
+      <c r="H10" s="0" t="n">
+        <v>99672</v>
+      </c>
+      <c r="I10" s="0" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B11" s="0" t="n">
-        <v>78.979</v>
+        <v>18.688</v>
       </c>
       <c r="C11" s="0" t="n">
-        <v>77.826</v>
+        <v>18.075</v>
       </c>
       <c r="D11" s="0" t="n">
-        <v>1.48</v>
+        <v>3.391</v>
       </c>
       <c r="E11" s="0" t="n">
-        <v>1486</v>
+        <v>331</v>
       </c>
       <c r="F11" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="0" t="s">
-        <v>19</v>
+      <c r="G11" s="0" t="n">
+        <v>510153</v>
+      </c>
+      <c r="H11" s="0" t="n">
+        <v>176000</v>
+      </c>
+      <c r="I11" s="0" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>